<commit_message>
Importación de Excel: nueva estructura (Fecha de Inicio MM/DD/AAAA, Idioma, Notas)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0145quBWM77zPaijQvdrjjMg
</commit_message>
<xml_diff>
--- a/public/plantilla_retiros.xlsx
+++ b/public/plantilla_retiros.xlsx
@@ -55,9 +55,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -423,16 +424,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="32" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -448,27 +451,37 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Lugar / Parroquia</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Fecha de Inicio</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Fechas</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Lugar / Parroquia</t>
-        </is>
-      </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>Idioma</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>Contacto</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Teléfono / Email</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Notas</t>
         </is>
       </c>
     </row>
@@ -485,27 +498,37 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>Parroquia San José</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>03/05/2027</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
           <t>Mujeres</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2027-03-05</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Parroquia San José</t>
-        </is>
-      </c>
       <c r="F2" t="inlineStr">
         <is>
+          <t>Español</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
           <t>María Gómez</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>300 123 4567 / maria@correo.com</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Cupos limitados</t>
         </is>
       </c>
     </row>
@@ -522,29 +545,35 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>St. James Church</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>05/14/2027</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
           <t>Hombres</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>12-14 de mayo de 2027</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>St. James Church</t>
-        </is>
-      </c>
       <c r="F3" t="inlineStr">
         <is>
+          <t>Inglés</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
           <t>Juan Pérez</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>407-555-1212</t>
         </is>
       </c>
+      <c r="I3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>